<commit_message>
Day 4 to Day 6 Excel practice completed
</commit_message>
<xml_diff>
--- a/Excel/Pinterest_Analytics_Project_Day3.xlsx
+++ b/Excel/Pinterest_Analytics_Project_Day3.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/afea116efc88aa0e/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/afea116efc88aa0e/Desktop/Pinterest-Analytics-Project/Excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="510" documentId="8_{4E26A75A-E90E-45A9-9012-17B855BCC5DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8901C23E-9C4E-4E65-AB46-F3E4CD8BAB6E}"/>
+  <xr:revisionPtr revIDLastSave="884" documentId="8_{4E26A75A-E90E-45A9-9012-17B855BCC5DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C4FFB35F-D012-42FC-8F00-6BDD851AA211}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="3" activeTab="6" xr2:uid="{7D575101-77E7-4AAE-AA6F-46947E88E8C0}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="8" activeTab="8" xr2:uid="{7D575101-77E7-4AAE-AA6F-46947E88E8C0}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,10 @@
     <sheet name="category_Analysis" sheetId="4" r:id="rId5"/>
     <sheet name="Hook_Analysis" sheetId="5" r:id="rId6"/>
     <sheet name="Dashboard" sheetId="6" r:id="rId7"/>
+    <sheet name="Day 4 practice" sheetId="8" r:id="rId8"/>
+    <sheet name="Day 6 vlookup" sheetId="9" r:id="rId9"/>
+    <sheet name="Hlookup" sheetId="10" r:id="rId10"/>
+    <sheet name="Xlookup" sheetId="12" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="148">
   <si>
     <t>A</t>
   </si>
@@ -309,13 +313,190 @@
   </si>
   <si>
     <t>Benefits</t>
+  </si>
+  <si>
+    <t>Impressions</t>
+  </si>
+  <si>
+    <t>Dish Rack</t>
+  </si>
+  <si>
+    <t>Spice Jar</t>
+  </si>
+  <si>
+    <t>Water Bottle</t>
+  </si>
+  <si>
+    <t>School</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kitchen </t>
+  </si>
+  <si>
+    <t>Perofrmance</t>
+  </si>
+  <si>
+    <t>Storage Container</t>
+  </si>
+  <si>
+    <t>How many pins have 1 impression?</t>
+  </si>
+  <si>
+    <t>How many pins are marked "Good"?</t>
+  </si>
+  <si>
+    <t>Total impressions from Home Organization category</t>
+  </si>
+  <si>
+    <t>Average impressions for school category</t>
+  </si>
+  <si>
+    <t>Count pins belong to school category</t>
+  </si>
+  <si>
+    <t>Count pins belong to Home Organization category</t>
+  </si>
+  <si>
+    <t>Find total impressions for Kitchen category</t>
+  </si>
+  <si>
+    <t>Find average impressions for Home Organization category.</t>
+  </si>
+  <si>
+    <t>count pins marked low</t>
+  </si>
+  <si>
+    <t>Pin ID</t>
+  </si>
+  <si>
+    <t>Pin Name</t>
+  </si>
+  <si>
+    <t>P101</t>
+  </si>
+  <si>
+    <t>P102</t>
+  </si>
+  <si>
+    <t>P103</t>
+  </si>
+  <si>
+    <t>P104</t>
+  </si>
+  <si>
+    <t>P105</t>
+  </si>
+  <si>
+    <t>School Bag</t>
+  </si>
+  <si>
+    <t>Bathroom Shelf</t>
+  </si>
+  <si>
+    <t>Kitchen Organization</t>
+  </si>
+  <si>
+    <t>Search Pin ID</t>
+  </si>
+  <si>
+    <t>Result</t>
+  </si>
+  <si>
+    <t>Impression</t>
+  </si>
+  <si>
+    <t>Pin.No</t>
+  </si>
+  <si>
+    <t>PinID</t>
+  </si>
+  <si>
+    <t>PinName</t>
+  </si>
+  <si>
+    <t>water Bottle</t>
+  </si>
+  <si>
+    <t>ProductID</t>
+  </si>
+  <si>
+    <t>ProductName</t>
+  </si>
+  <si>
+    <t>Price</t>
+  </si>
+  <si>
+    <t>P1001</t>
+  </si>
+  <si>
+    <t>P1002</t>
+  </si>
+  <si>
+    <t>P1003</t>
+  </si>
+  <si>
+    <t>P1004</t>
+  </si>
+  <si>
+    <t>P1005</t>
+  </si>
+  <si>
+    <t>Pen</t>
+  </si>
+  <si>
+    <t>USB Cable</t>
+  </si>
+  <si>
+    <t>Mouse</t>
+  </si>
+  <si>
+    <t>Stationery</t>
+  </si>
+  <si>
+    <t>Electronics</t>
+  </si>
+  <si>
+    <t>Lifestyle</t>
+  </si>
+  <si>
+    <t>Product ID</t>
+  </si>
+  <si>
+    <t>Qty</t>
+  </si>
+  <si>
+    <t>OrderID</t>
+  </si>
+  <si>
+    <t>O-001</t>
+  </si>
+  <si>
+    <t>O-002</t>
+  </si>
+  <si>
+    <t>O-003</t>
+  </si>
+  <si>
+    <t>O-004</t>
+  </si>
+  <si>
+    <t>O-005</t>
+  </si>
+  <si>
+    <t>Ordered ProductName</t>
+  </si>
+  <si>
+    <t>Note Book</t>
+  </si>
+  <si>
+    <t>P999</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -378,8 +559,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="16">
+  <fills count="20">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -470,8 +657,32 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="16">
+  <borders count="24">
     <border>
       <left/>
       <right/>
@@ -698,11 +909,105 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -773,15 +1078,6 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -794,12 +1090,6 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -810,10 +1100,40 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="15" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -828,6 +1148,9 @@
     <xf numFmtId="0" fontId="2" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -840,17 +1163,52 @@
     <xf numFmtId="0" fontId="2" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="21" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="22" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="23" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="23">
     <dxf>
       <font>
         <color rgb="FF9C5700"/>
@@ -907,6 +1265,301 @@
           <bgColor theme="9"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+      </border>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -4464,6 +5117,44 @@
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{7C454B97-C1F5-4F5F-B5EE-AC02F7B74478}" name="Table4" displayName="Table4" ref="A1:C6" totalsRowShown="0" headerRowDxfId="6" headerRowBorderDxfId="11" tableBorderDxfId="12" totalsRowBorderDxfId="10">
+  <autoFilter ref="A1:C6" xr:uid="{7C454B97-C1F5-4F5F-B5EE-AC02F7B74478}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{3E6477C8-2135-4B84-8319-42F859D90507}" name="Pin ID" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{F73159FA-823A-4F43-A70E-984D5F1F61EC}" name="Pin Name" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{3543AFAF-EE44-4BF0-9040-BE9037A4BBB6}" name="Category" dataDxfId="7"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{EEBD6B94-D2AF-4094-B371-0CF79DA4513E}" name="Table2" displayName="Table2" ref="A1:E3" totalsRowShown="0" headerRowDxfId="13" dataDxfId="14" headerRowBorderDxfId="21" tableBorderDxfId="22" totalsRowBorderDxfId="20">
+  <autoFilter ref="A1:E3" xr:uid="{EEBD6B94-D2AF-4094-B371-0CF79DA4513E}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{F1C14BA4-8880-44D3-A737-43854E2C01A7}" name="Pin.No" dataDxfId="19"/>
+    <tableColumn id="2" xr3:uid="{312251DA-CCF9-41CA-A98C-6FE29825011F}" name="P101" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{E1D013AC-8688-4EAB-8813-5C5B89991004}" name="P102" dataDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{14579D8A-F53C-432B-AEC4-3AB7418C02EB}" name="P103" dataDxfId="16"/>
+    <tableColumn id="5" xr3:uid="{6E847491-C0B0-4C45-8588-CD26A20A409B}" name="P104" dataDxfId="15"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{26F8B813-0CE2-4AA9-B32C-B497FB2649A9}" name="Table5" displayName="Table5" ref="A1:C6" totalsRowShown="0">
+  <autoFilter ref="A1:C6" xr:uid="{26F8B813-0CE2-4AA9-B32C-B497FB2649A9}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{BC95DD1B-B955-4803-95A6-BD466FCE9456}" name="PinID"/>
+    <tableColumn id="2" xr3:uid="{A0E5B7D0-6DE7-48DD-B860-9075F8C25FC3}" name="PinName"/>
+    <tableColumn id="3" xr3:uid="{ED963EFA-F23A-4261-A72F-8A058AAAB554}" name="Category"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -4864,6 +5555,179 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5863D121-28B4-4596-B926-D7E386D7861C}">
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.90625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" s="60" t="s">
+        <v>119</v>
+      </c>
+      <c r="B1" s="61" t="s">
+        <v>108</v>
+      </c>
+      <c r="C1" s="61" t="s">
+        <v>109</v>
+      </c>
+      <c r="D1" s="61" t="s">
+        <v>110</v>
+      </c>
+      <c r="E1" s="62" t="s">
+        <v>111</v>
+      </c>
+      <c r="F1" s="8"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" s="58" t="s">
+        <v>107</v>
+      </c>
+      <c r="B2" s="57" t="s">
+        <v>113</v>
+      </c>
+      <c r="C2" s="57" t="s">
+        <v>114</v>
+      </c>
+      <c r="D2" s="57" t="s">
+        <v>90</v>
+      </c>
+      <c r="E2" s="59" t="s">
+        <v>55</v>
+      </c>
+      <c r="F2" s="8"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" s="63" t="s">
+        <v>118</v>
+      </c>
+      <c r="B3" s="64">
+        <v>3</v>
+      </c>
+      <c r="C3" s="64">
+        <v>3</v>
+      </c>
+      <c r="D3" s="64">
+        <v>2</v>
+      </c>
+      <c r="E3" s="65">
+        <v>1</v>
+      </c>
+      <c r="F3" s="8"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>110</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="8" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{996B43B9-90F3-4FF9-9A31-FF1693A4A3C8}">
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="7.36328125" customWidth="1"/>
+    <col min="2" max="2" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.7265625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C2" t="s">
+        <v>113</v>
+      </c>
+      <c r="E2" t="s">
+        <v>110</v>
+      </c>
+      <c r="F2" t="str">
+        <f>_xlfn.XLOOKUP(E2,A2:A6,B2:B6)</f>
+        <v>Dish Rack</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>109</v>
+      </c>
+      <c r="B3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>110</v>
+      </c>
+      <c r="B4" t="s">
+        <v>90</v>
+      </c>
+      <c r="C4" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>111</v>
+      </c>
+      <c r="B5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C6" t="s">
+        <v>122</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="8" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6D11031-D0DD-4C34-B7C4-D60CD9947AD2}">
   <dimension ref="A1:F25"/>
@@ -4878,14 +5742,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="26"/>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="42"/>
     </row>
     <row r="2" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
@@ -5436,73 +6300,73 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="34" t="s">
         <v>83</v>
       </c>
-      <c r="B1" s="49" t="s">
+      <c r="B1" s="34" t="s">
         <v>45</v>
       </c>
       <c r="C1" s="8"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" s="50" t="s">
+      <c r="A2" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="B2" s="50">
+      <c r="B2" s="35">
         <v>20</v>
       </c>
       <c r="C2" s="8"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="B3" s="50">
+      <c r="B3" s="35">
         <v>27</v>
       </c>
       <c r="C3" s="8"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" s="50" t="s">
+      <c r="A4" s="35" t="s">
         <v>48</v>
       </c>
-      <c r="B4" s="50">
+      <c r="B4" s="35">
         <v>1.35</v>
       </c>
       <c r="C4" s="8"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" s="50" t="s">
+      <c r="A5" s="35" t="s">
         <v>84</v>
       </c>
-      <c r="B5" s="50" t="s">
+      <c r="B5" s="35" t="s">
         <v>52</v>
       </c>
       <c r="C5" s="8"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" s="50" t="s">
+      <c r="A6" s="35" t="s">
         <v>85</v>
       </c>
-      <c r="B6" s="50" t="s">
+      <c r="B6" s="35" t="s">
         <v>88</v>
       </c>
       <c r="C6" s="8"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A7" s="50" t="s">
+      <c r="A7" s="35" t="s">
         <v>86</v>
       </c>
-      <c r="B7" s="50" t="s">
+      <c r="B7" s="35" t="s">
         <v>23</v>
       </c>
       <c r="C7" s="8"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A8" s="50" t="s">
+      <c r="A8" s="35" t="s">
         <v>87</v>
       </c>
-      <c r="B8" s="50">
+      <c r="B8" s="35">
         <v>3</v>
       </c>
       <c r="C8" s="8"/>
@@ -5527,10 +6391,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="26" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="28" t="s">
+      <c r="B1" s="25" t="s">
         <v>20</v>
       </c>
     </row>
@@ -5632,57 +6496,57 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="18.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="27" t="s">
         <v>60</v>
       </c>
-      <c r="B1" s="30" t="s">
+      <c r="B1" s="27" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="29" t="s">
+      <c r="A2" s="26" t="s">
         <v>62</v>
       </c>
-      <c r="B2" s="29">
+      <c r="B2" s="26">
         <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="26" t="s">
         <v>63</v>
       </c>
-      <c r="B3" s="29">
+      <c r="B3" s="26">
         <v>8</v>
       </c>
-      <c r="D3" s="31" t="s">
+      <c r="D3" s="43" t="s">
         <v>69</v>
       </c>
-      <c r="E3" s="32"/>
-      <c r="F3" s="32"/>
-      <c r="G3" s="32"/>
-      <c r="H3" s="32"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="44"/>
+      <c r="G3" s="44"/>
+      <c r="H3" s="44"/>
     </row>
     <row r="4" spans="1:8" ht="21.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="29" t="s">
+      <c r="A4" s="26" t="s">
         <v>64</v>
       </c>
-      <c r="B4" s="29">
+      <c r="B4" s="26">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="26" t="s">
         <v>65</v>
       </c>
-      <c r="B5" s="29">
+      <c r="B5" s="26">
         <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="29" t="s">
+      <c r="A6" s="26" t="s">
         <v>66</v>
       </c>
-      <c r="B6" s="29">
+      <c r="B6" s="26">
         <v>2</v>
       </c>
     </row>
@@ -5736,117 +6600,117 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="22" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="34" t="s">
+      <c r="B1" s="29" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="21" x14ac:dyDescent="0.5">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="30" t="s">
         <v>71</v>
       </c>
-      <c r="B2" s="36">
+      <c r="B2" s="31">
         <f>SUM('Performance overview'!B2)</f>
         <v>20</v>
       </c>
-      <c r="G2" s="39" t="s">
+      <c r="G2" s="45" t="s">
         <v>75</v>
       </c>
-      <c r="H2" s="39"/>
-      <c r="I2" s="39"/>
-      <c r="J2" s="39"/>
-      <c r="K2" s="39"/>
-      <c r="O2" s="41" t="s">
+      <c r="H2" s="45"/>
+      <c r="I2" s="45"/>
+      <c r="J2" s="45"/>
+      <c r="K2" s="45"/>
+      <c r="O2" s="46" t="s">
         <v>77</v>
       </c>
-      <c r="P2" s="42"/>
-      <c r="Q2" s="42"/>
-      <c r="R2" s="42"/>
-      <c r="S2" s="43"/>
+      <c r="P2" s="47"/>
+      <c r="Q2" s="47"/>
+      <c r="R2" s="47"/>
+      <c r="S2" s="48"/>
     </row>
     <row r="3" spans="1:19" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A3" s="35" t="s">
+      <c r="A3" s="30" t="s">
         <v>72</v>
       </c>
-      <c r="B3" s="36">
+      <c r="B3" s="31">
         <f>SUM('Performance overview'!B3)</f>
         <v>27</v>
       </c>
-      <c r="O3" s="44" t="s">
+      <c r="O3" s="49" t="s">
         <v>78</v>
       </c>
-      <c r="P3" s="40"/>
-      <c r="Q3" s="40"/>
-      <c r="R3" s="40"/>
-      <c r="S3" s="45"/>
+      <c r="P3" s="50"/>
+      <c r="Q3" s="50"/>
+      <c r="R3" s="50"/>
+      <c r="S3" s="51"/>
     </row>
     <row r="4" spans="1:19" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A4" s="35" t="s">
+      <c r="A4" s="30" t="s">
         <v>73</v>
       </c>
-      <c r="B4" s="36">
+      <c r="B4" s="31">
         <f>MAX(category_Analysis!A1:C10)</f>
         <v>9</v>
       </c>
-      <c r="O4" s="44" t="s">
+      <c r="O4" s="49" t="s">
         <v>79</v>
       </c>
-      <c r="P4" s="40"/>
-      <c r="Q4" s="40"/>
-      <c r="R4" s="40"/>
-      <c r="S4" s="45"/>
+      <c r="P4" s="50"/>
+      <c r="Q4" s="50"/>
+      <c r="R4" s="50"/>
+      <c r="S4" s="51"/>
     </row>
     <row r="5" spans="1:19" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A5" s="35" t="s">
+      <c r="A5" s="30" t="s">
         <v>68</v>
       </c>
-      <c r="B5" s="36">
+      <c r="B5" s="31">
         <f>MAX(Hook_Analysis!A1:B6)</f>
         <v>10</v>
       </c>
-      <c r="O5" s="44" t="s">
+      <c r="O5" s="49" t="s">
         <v>80</v>
       </c>
-      <c r="P5" s="40"/>
-      <c r="Q5" s="40"/>
-      <c r="R5" s="40"/>
-      <c r="S5" s="45"/>
+      <c r="P5" s="50"/>
+      <c r="Q5" s="50"/>
+      <c r="R5" s="50"/>
+      <c r="S5" s="51"/>
     </row>
     <row r="6" spans="1:19" ht="19" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A6" s="37" t="s">
+      <c r="A6" s="32" t="s">
         <v>74</v>
       </c>
-      <c r="B6" s="38">
+      <c r="B6" s="33">
         <f>AVERAGE('Performance overview'!B4)</f>
         <v>1.35</v>
       </c>
-      <c r="O6" s="44" t="s">
+      <c r="O6" s="49" t="s">
         <v>81</v>
       </c>
-      <c r="P6" s="40"/>
-      <c r="Q6" s="40"/>
-      <c r="R6" s="40"/>
-      <c r="S6" s="45"/>
+      <c r="P6" s="50"/>
+      <c r="Q6" s="50"/>
+      <c r="R6" s="50"/>
+      <c r="S6" s="51"/>
     </row>
     <row r="7" spans="1:19" ht="19" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="O7" s="46" t="s">
+      <c r="O7" s="52" t="s">
         <v>82</v>
       </c>
-      <c r="P7" s="47"/>
-      <c r="Q7" s="47"/>
-      <c r="R7" s="47"/>
-      <c r="S7" s="48"/>
+      <c r="P7" s="53"/>
+      <c r="Q7" s="53"/>
+      <c r="R7" s="53"/>
+      <c r="S7" s="54"/>
     </row>
     <row r="22" spans="7:11" ht="21" x14ac:dyDescent="0.5">
-      <c r="G22" s="39" t="s">
+      <c r="G22" s="45" t="s">
         <v>76</v>
       </c>
-      <c r="H22" s="39"/>
-      <c r="I22" s="39"/>
-      <c r="J22" s="39"/>
-      <c r="K22" s="39"/>
+      <c r="H22" s="45"/>
+      <c r="I22" s="45"/>
+      <c r="J22" s="45"/>
+      <c r="K22" s="45"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -5862,4 +6726,523 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E75E8015-A1D8-4F75-A9BA-5D044AEC3F30}">
+  <dimension ref="A1:D24"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="4" width="21.1796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="18.5" x14ac:dyDescent="0.35">
+      <c r="A1" s="36" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="36" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="36" t="s">
+        <v>89</v>
+      </c>
+      <c r="D1" s="38" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="37" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" s="37" t="s">
+        <v>93</v>
+      </c>
+      <c r="C2" s="37">
+        <v>3</v>
+      </c>
+      <c r="D2" s="37" t="str">
+        <f>IF(C2&gt;=2,"Good","Low")</f>
+        <v>Good</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="37" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="37" t="s">
+        <v>52</v>
+      </c>
+      <c r="C3" s="37">
+        <v>3</v>
+      </c>
+      <c r="D3" s="37" t="str">
+        <f t="shared" ref="D3:D9" si="0">IF(C3&gt;=2,"Good","Low")</f>
+        <v>Good</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="37" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="37" t="s">
+        <v>53</v>
+      </c>
+      <c r="C4" s="37">
+        <v>2</v>
+      </c>
+      <c r="D4" s="37" t="str">
+        <f t="shared" si="0"/>
+        <v>Good</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="37" t="s">
+        <v>90</v>
+      </c>
+      <c r="B5" s="37" t="s">
+        <v>52</v>
+      </c>
+      <c r="C5" s="37">
+        <v>2</v>
+      </c>
+      <c r="D5" s="37" t="str">
+        <f t="shared" si="0"/>
+        <v>Good</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="37" t="s">
+        <v>91</v>
+      </c>
+      <c r="B6" s="37" t="s">
+        <v>94</v>
+      </c>
+      <c r="C6" s="37">
+        <v>2</v>
+      </c>
+      <c r="D6" s="37" t="str">
+        <f t="shared" si="0"/>
+        <v>Good</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="37" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="37" t="s">
+        <v>93</v>
+      </c>
+      <c r="C7" s="37">
+        <v>1</v>
+      </c>
+      <c r="D7" s="37" t="str">
+        <f t="shared" si="0"/>
+        <v>Low</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="37" t="s">
+        <v>96</v>
+      </c>
+      <c r="B8" s="37" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="37">
+        <v>1</v>
+      </c>
+      <c r="D8" s="37" t="str">
+        <f t="shared" si="0"/>
+        <v>Low</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="37" t="s">
+        <v>92</v>
+      </c>
+      <c r="B9" s="37" t="s">
+        <v>93</v>
+      </c>
+      <c r="C9" s="37">
+        <v>1</v>
+      </c>
+      <c r="D9" s="37" t="str">
+        <f t="shared" si="0"/>
+        <v>Low</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="39" t="s">
+        <v>97</v>
+      </c>
+      <c r="B13" s="39"/>
+      <c r="C13">
+        <f>COUNTIF(C2:C9,1)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="39" t="s">
+        <v>98</v>
+      </c>
+      <c r="B14" s="39"/>
+      <c r="C14">
+        <f>COUNTIF(D2:D9,"Good")</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="39" t="s">
+        <v>99</v>
+      </c>
+      <c r="B15" s="39"/>
+      <c r="C15">
+        <f>(SUMIF(B2:B9,"Home Organization",C2:C9))</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" s="39" t="s">
+        <v>100</v>
+      </c>
+      <c r="B16" s="39"/>
+      <c r="C16">
+        <f>AVERAGEIF(B2:B9,"School",C2:C9)</f>
+        <v>1.6666666666666667</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A20" s="39" t="s">
+        <v>101</v>
+      </c>
+      <c r="B20" s="39"/>
+      <c r="C20">
+        <f>COUNTIF(B2:B9,"School")</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A21" s="39" t="s">
+        <v>102</v>
+      </c>
+      <c r="B21" s="39"/>
+      <c r="C21">
+        <f>COUNTIF(B2:B9,"Home Organization")</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A22" s="39" t="s">
+        <v>103</v>
+      </c>
+      <c r="B22" s="39"/>
+      <c r="C22">
+        <f>SUMIF(B2:B9,"Kitchen",C2:C9)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A23" s="39" t="s">
+        <v>104</v>
+      </c>
+      <c r="B23" s="39"/>
+      <c r="C23">
+        <f>AVERAGEIF(B2:B9,"Home Organization",C2:C9)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A24" s="39" t="s">
+        <v>105</v>
+      </c>
+      <c r="B24" s="39"/>
+      <c r="C24">
+        <f>COUNTIF(D2:D9,"low")</f>
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A21:B21"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16DA3542-98D2-41F0-A62F-F7003BBA945E}">
+  <dimension ref="A1:F25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="4" width="19.1796875" customWidth="1"/>
+    <col min="5" max="5" width="11.81640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" s="66" t="s">
+        <v>106</v>
+      </c>
+      <c r="B1" s="67" t="s">
+        <v>107</v>
+      </c>
+      <c r="C1" s="68" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" s="55" t="s">
+        <v>116</v>
+      </c>
+      <c r="F1" s="55" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" s="69" t="s">
+        <v>108</v>
+      </c>
+      <c r="B2" s="70" t="s">
+        <v>113</v>
+      </c>
+      <c r="C2" s="71" t="s">
+        <v>113</v>
+      </c>
+      <c r="E2" s="56" t="s">
+        <v>112</v>
+      </c>
+      <c r="F2" t="str">
+        <f>VLOOKUP(E2,A2:C6,3,FALSE)</f>
+        <v>Water Bottle</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" s="69" t="s">
+        <v>109</v>
+      </c>
+      <c r="B3" s="70" t="s">
+        <v>114</v>
+      </c>
+      <c r="C3" s="71" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" s="69" t="s">
+        <v>110</v>
+      </c>
+      <c r="B4" s="70" t="s">
+        <v>90</v>
+      </c>
+      <c r="C4" s="71" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" s="69" t="s">
+        <v>111</v>
+      </c>
+      <c r="B5" s="70" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="71" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" s="72" t="s">
+        <v>112</v>
+      </c>
+      <c r="B6" s="73" t="s">
+        <v>92</v>
+      </c>
+      <c r="C6" s="74" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" s="75" t="s">
+        <v>123</v>
+      </c>
+      <c r="B10" s="75" t="s">
+        <v>124</v>
+      </c>
+      <c r="C10" s="75" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" s="75" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="D11" s="8">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="D12" s="8">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="D13" s="8">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="D14" s="8">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="D15" s="8">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" s="75" t="s">
+        <v>139</v>
+      </c>
+      <c r="B20" s="75" t="s">
+        <v>137</v>
+      </c>
+      <c r="C20" s="75" t="s">
+        <v>138</v>
+      </c>
+      <c r="D20" s="75" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>140</v>
+      </c>
+      <c r="B21" t="s">
+        <v>128</v>
+      </c>
+      <c r="C21">
+        <v>2</v>
+      </c>
+      <c r="D21" t="str">
+        <f t="shared" ref="D21:D25" si="0">IFERROR(VLOOKUP(B17,$A$12:$D$16,2,FALSE),"Product Not Found")</f>
+        <v>Product Not Found</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>141</v>
+      </c>
+      <c r="B22" t="s">
+        <v>126</v>
+      </c>
+      <c r="C22">
+        <v>5</v>
+      </c>
+      <c r="D22" t="str">
+        <f t="shared" si="0"/>
+        <v>Product Not Found</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>142</v>
+      </c>
+      <c r="B23" t="s">
+        <v>129</v>
+      </c>
+      <c r="C23">
+        <v>1</v>
+      </c>
+      <c r="D23" t="str">
+        <f t="shared" si="0"/>
+        <v>Product Not Found</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>143</v>
+      </c>
+      <c r="B24" t="s">
+        <v>127</v>
+      </c>
+      <c r="C24">
+        <v>10</v>
+      </c>
+      <c r="D24" t="str">
+        <f t="shared" si="0"/>
+        <v>Product Not Found</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>144</v>
+      </c>
+      <c r="B25" t="s">
+        <v>147</v>
+      </c>
+      <c r="C25">
+        <v>1</v>
+      </c>
+      <c r="D25" t="str">
+        <f t="shared" si="0"/>
+        <v>USB Cable</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="8" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
xlookup, text to columns,remove duplicates
</commit_message>
<xml_diff>
--- a/Excel/Pinterest_Analytics_Project_Day3.xlsx
+++ b/Excel/Pinterest_Analytics_Project_Day3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/afea116efc88aa0e/Desktop/Pinterest-Analytics-Project/Excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1001" documentId="8_{4E26A75A-E90E-45A9-9012-17B855BCC5DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F72FC9A1-A4FC-42F2-B8B4-2BDEDC851D53}"/>
+  <xr:revisionPtr revIDLastSave="1076" documentId="8_{4E26A75A-E90E-45A9-9012-17B855BCC5DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1D845077-E52A-413A-A6D2-84416642E3C5}"/>
   <bookViews>
-    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" firstSheet="9" activeTab="10" xr2:uid="{7D575101-77E7-4AAE-AA6F-46947E88E8C0}"/>
+    <workbookView minimized="1" xWindow="680" yWindow="680" windowWidth="7500" windowHeight="6000" activeTab="1" xr2:uid="{7D575101-77E7-4AAE-AA6F-46947E88E8C0}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,12 @@
     <sheet name=" vlookup " sheetId="13" r:id="rId9"/>
     <sheet name="HLookUp" sheetId="14" r:id="rId10"/>
     <sheet name="xlookup" sheetId="15" r:id="rId11"/>
+    <sheet name="Text to Columns" sheetId="16" r:id="rId12"/>
+    <sheet name="Remove duplicates" sheetId="17" r:id="rId13"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Raw_Data!$A$2:$F$22</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -46,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="141">
   <si>
     <t>A</t>
   </si>
@@ -135,9 +140,6 @@
     <t>Lunch bag</t>
   </si>
   <si>
-    <t>storage container</t>
-  </si>
-  <si>
     <t>Storage Baskets</t>
   </si>
   <si>
@@ -430,6 +432,48 @@
   </si>
   <si>
     <t>other product</t>
+  </si>
+  <si>
+    <t>P9999</t>
+  </si>
+  <si>
+    <t>Rekha</t>
+  </si>
+  <si>
+    <t>Hyderabad</t>
+  </si>
+  <si>
+    <t>India</t>
+  </si>
+  <si>
+    <t>Anu</t>
+  </si>
+  <si>
+    <t>Bengaluru</t>
+  </si>
+  <si>
+    <t>Priya</t>
+  </si>
+  <si>
+    <t>Chennai</t>
+  </si>
+  <si>
+    <t>Rahul</t>
+  </si>
+  <si>
+    <t>Mumbai</t>
+  </si>
+  <si>
+    <t>Ravi</t>
+  </si>
+  <si>
+    <t>Delhi</t>
+  </si>
+  <si>
+    <t>School Bag</t>
+  </si>
+  <si>
+    <t>foldable drawer organizer</t>
   </si>
 </sst>
 </file>
@@ -864,7 +908,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -972,6 +1016,57 @@
     <xf numFmtId="0" fontId="3" fillId="16" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1020,56 +1115,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5099,100 +5146,100 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="56" t="s">
+      <c r="A1" s="40" t="s">
+        <v>115</v>
+      </c>
+      <c r="B1" s="43" t="s">
+        <v>106</v>
+      </c>
+      <c r="C1" s="43" t="s">
+        <v>107</v>
+      </c>
+      <c r="D1" s="43" t="s">
+        <v>108</v>
+      </c>
+      <c r="E1" s="43" t="s">
+        <v>109</v>
+      </c>
+      <c r="F1" s="43" t="s">
+        <v>110</v>
+      </c>
+      <c r="G1" s="45" t="s">
         <v>116</v>
       </c>
-      <c r="B1" s="59" t="s">
-        <v>107</v>
-      </c>
-      <c r="C1" s="59" t="s">
-        <v>108</v>
-      </c>
-      <c r="D1" s="59" t="s">
-        <v>109</v>
-      </c>
-      <c r="E1" s="59" t="s">
-        <v>110</v>
-      </c>
-      <c r="F1" s="59" t="s">
+    </row>
+    <row r="2" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="41" t="s">
+        <v>117</v>
+      </c>
+      <c r="B2" s="39" t="s">
+        <v>119</v>
+      </c>
+      <c r="C2" s="39" t="s">
+        <v>120</v>
+      </c>
+      <c r="D2" s="39" t="s">
         <v>111</v>
       </c>
-      <c r="G1" s="61" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="57" t="s">
+      <c r="E2" s="39" t="s">
+        <v>112</v>
+      </c>
+      <c r="F2" s="39" t="s">
+        <v>121</v>
+      </c>
+      <c r="G2" s="46" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="41" t="s">
+        <v>105</v>
+      </c>
+      <c r="B3" s="39">
+        <v>80</v>
+      </c>
+      <c r="C3" s="39">
+        <v>120</v>
+      </c>
+      <c r="D3" s="39">
+        <v>250</v>
+      </c>
+      <c r="E3" s="39">
+        <v>600</v>
+      </c>
+      <c r="F3" s="39">
+        <v>450</v>
+      </c>
+      <c r="G3" s="46">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="42" t="s">
         <v>118</v>
       </c>
-      <c r="B2" s="55" t="s">
-        <v>120</v>
-      </c>
-      <c r="C2" s="55" t="s">
-        <v>121</v>
-      </c>
-      <c r="D2" s="55" t="s">
-        <v>112</v>
-      </c>
-      <c r="E2" s="55" t="s">
-        <v>113</v>
-      </c>
-      <c r="F2" s="55" t="s">
-        <v>122</v>
-      </c>
-      <c r="G2" s="62" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="57" t="s">
-        <v>106</v>
-      </c>
-      <c r="B3" s="55">
-        <v>80</v>
-      </c>
-      <c r="C3" s="55">
-        <v>120</v>
-      </c>
-      <c r="D3" s="55">
-        <v>250</v>
-      </c>
-      <c r="E3" s="55">
-        <v>600</v>
-      </c>
-      <c r="F3" s="55">
-        <v>450</v>
-      </c>
-      <c r="G3" s="62">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="58" t="s">
-        <v>119</v>
-      </c>
-      <c r="B4" s="60">
+      <c r="B4" s="44">
         <v>25</v>
       </c>
-      <c r="C4" s="60">
+      <c r="C4" s="44">
         <v>40</v>
       </c>
-      <c r="D4" s="60">
+      <c r="D4" s="44">
         <v>15</v>
       </c>
-      <c r="E4" s="60">
+      <c r="E4" s="44">
         <v>10</v>
       </c>
-      <c r="F4" s="60">
+      <c r="F4" s="44">
         <v>20</v>
       </c>
-      <c r="G4" s="63">
+      <c r="G4" s="47">
         <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" s="64" t="s">
-        <v>126</v>
+      <c r="A6" s="48" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
@@ -5227,35 +5274,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A1" s="65" t="s">
-        <v>116</v>
-      </c>
-      <c r="B1" s="66" t="s">
+      <c r="A1" s="49" t="s">
+        <v>115</v>
+      </c>
+      <c r="B1" s="50" t="s">
+        <v>117</v>
+      </c>
+      <c r="C1" s="50" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="50" t="s">
+        <v>105</v>
+      </c>
+      <c r="E1" s="51" t="s">
         <v>118</v>
       </c>
-      <c r="C1" s="66" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1" s="66" t="s">
+      <c r="F1" s="8"/>
+      <c r="G1" s="52" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A2" s="53" t="s">
         <v>106</v>
       </c>
-      <c r="E1" s="67" t="s">
+      <c r="B2" s="35" t="s">
         <v>119</v>
       </c>
-      <c r="F1" s="8"/>
-      <c r="G1" s="68" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" s="69" t="s">
-        <v>107</v>
-      </c>
-      <c r="B2" s="35" t="s">
-        <v>120</v>
-      </c>
       <c r="C2" s="35" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D2" s="35">
         <v>80</v>
@@ -5270,14 +5317,14 @@
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" s="69" t="s">
-        <v>108</v>
+      <c r="A3" s="53" t="s">
+        <v>107</v>
       </c>
       <c r="B3" s="35" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C3" s="35" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D3" s="35">
         <v>120</v>
@@ -5286,17 +5333,20 @@
         <v>40</v>
       </c>
       <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
+      <c r="G3" s="8" t="str">
+        <f>_xlfn.XLOOKUP(A4,A2:A7,C2:C7)</f>
+        <v>Electronics</v>
+      </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" s="69" t="s">
-        <v>109</v>
+      <c r="A4" s="53" t="s">
+        <v>108</v>
       </c>
       <c r="B4" s="35" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C4" s="35" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D4" s="35">
         <v>250</v>
@@ -5305,17 +5355,20 @@
         <v>15</v>
       </c>
       <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
+      <c r="G4" s="8">
+        <f>_xlfn.XLOOKUP(A7,A2:A7,D2:D7)</f>
+        <v>300</v>
+      </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5" s="69" t="s">
-        <v>110</v>
+      <c r="A5" s="53" t="s">
+        <v>109</v>
       </c>
       <c r="B5" s="35" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C5" s="35" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D5" s="35">
         <v>600</v>
@@ -5324,17 +5377,20 @@
         <v>10</v>
       </c>
       <c r="F5" s="8"/>
-      <c r="G5" s="8"/>
+      <c r="G5" s="8">
+        <f>_xlfn.XLOOKUP(A3,A2:A7,E2:E7)</f>
+        <v>40</v>
+      </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" s="69" t="s">
-        <v>111</v>
+      <c r="A6" s="53" t="s">
+        <v>110</v>
       </c>
       <c r="B6" s="35" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C6" s="35" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D6" s="35">
         <v>450</v>
@@ -5343,35 +5399,148 @@
         <v>20</v>
       </c>
       <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
+      <c r="G6" s="8" t="str">
+        <f>_xlfn.XLOOKUP(B5,B2:B7,C2:C7,"Product Not Found")</f>
+        <v>Electronics</v>
+      </c>
     </row>
     <row r="7" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="70" t="s">
-        <v>117</v>
-      </c>
-      <c r="B7" s="71" t="s">
-        <v>92</v>
-      </c>
-      <c r="C7" s="71" t="s">
-        <v>124</v>
-      </c>
-      <c r="D7" s="71">
+      <c r="A7" s="54" t="s">
+        <v>116</v>
+      </c>
+      <c r="B7" s="55" t="s">
+        <v>91</v>
+      </c>
+      <c r="C7" s="55" t="s">
+        <v>123</v>
+      </c>
+      <c r="D7" s="55">
         <v>300</v>
       </c>
       <c r="E7" s="23">
         <v>30</v>
       </c>
       <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
+      <c r="G7" s="8" t="str">
+        <f>_xlfn.XLOOKUP(A8,A2:A7,B2:B7,"product not found")</f>
+        <v>product not found</v>
+      </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A8" s="8"/>
+      <c r="A8" s="8" t="s">
+        <v>127</v>
+      </c>
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
       <c r="D8" s="8"/>
       <c r="E8" s="8"/>
       <c r="F8" s="8"/>
       <c r="G8" s="8"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DB47587-7068-43A7-B408-060824C950A4}">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="5.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.7265625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B2" t="s">
+        <v>132</v>
+      </c>
+      <c r="C2" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>133</v>
+      </c>
+      <c r="B3" t="s">
+        <v>134</v>
+      </c>
+      <c r="C3" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B4" t="s">
+        <v>136</v>
+      </c>
+      <c r="C4" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>137</v>
+      </c>
+      <c r="B5" t="s">
+        <v>138</v>
+      </c>
+      <c r="C5" t="s">
+        <v>130</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4C75690-6AEE-4F6E-A031-73756030F043}">
+  <dimension ref="A1:A5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1" s="72" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>112</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5392,14 +5561,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="56" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="41"/>
+      <c r="B1" s="57"/>
+      <c r="C1" s="57"/>
+      <c r="D1" s="57"/>
+      <c r="E1" s="57"/>
+      <c r="F1" s="58"/>
     </row>
     <row r="2" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
@@ -5409,7 +5578,7 @@
         <v>17</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>18</v>
@@ -5432,10 +5601,10 @@
         <v>23</v>
       </c>
       <c r="D3" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="E3" s="9" t="s">
         <v>42</v>
-      </c>
-      <c r="E3" s="9" t="s">
-        <v>43</v>
       </c>
       <c r="F3" s="10">
         <v>3</v>
@@ -5449,13 +5618,13 @@
         <v>24</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D4" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="E4" s="9" t="s">
         <v>42</v>
-      </c>
-      <c r="E4" s="9" t="s">
-        <v>43</v>
       </c>
       <c r="F4" s="10">
         <v>3</v>
@@ -5469,13 +5638,13 @@
         <v>25</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D5" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="E5" s="9" t="s">
         <v>42</v>
-      </c>
-      <c r="E5" s="9" t="s">
-        <v>43</v>
       </c>
       <c r="F5" s="10">
         <v>2</v>
@@ -5489,13 +5658,13 @@
         <v>26</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D6" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="E6" s="9" t="s">
         <v>42</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>43</v>
       </c>
       <c r="F6" s="10">
         <v>2</v>
@@ -5509,13 +5678,13 @@
         <v>27</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D7" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="E7" s="9" t="s">
         <v>42</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>43</v>
       </c>
       <c r="F7" s="10">
         <v>2</v>
@@ -5529,13 +5698,13 @@
         <v>28</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D8" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="E8" s="9" t="s">
         <v>42</v>
-      </c>
-      <c r="E8" s="9" t="s">
-        <v>43</v>
       </c>
       <c r="F8" s="10">
         <v>1</v>
@@ -5546,16 +5715,16 @@
         <v>7</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>29</v>
+        <v>140</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D9" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="E9" s="9" t="s">
         <v>42</v>
-      </c>
-      <c r="E9" s="9" t="s">
-        <v>43</v>
       </c>
       <c r="F9" s="10">
         <v>1</v>
@@ -5566,16 +5735,16 @@
         <v>8</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D10" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="E10" s="9" t="s">
         <v>42</v>
-      </c>
-      <c r="E10" s="9" t="s">
-        <v>43</v>
       </c>
       <c r="F10" s="10">
         <v>1</v>
@@ -5586,16 +5755,16 @@
         <v>9</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D11" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="E11" s="9" t="s">
         <v>42</v>
-      </c>
-      <c r="E11" s="9" t="s">
-        <v>43</v>
       </c>
       <c r="F11" s="10">
         <v>1</v>
@@ -5606,16 +5775,16 @@
         <v>10</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D12" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="E12" s="9" t="s">
         <v>42</v>
-      </c>
-      <c r="E12" s="9" t="s">
-        <v>43</v>
       </c>
       <c r="F12" s="10">
         <v>1</v>
@@ -5626,16 +5795,16 @@
         <v>11</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D13" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="E13" s="9" t="s">
         <v>42</v>
-      </c>
-      <c r="E13" s="9" t="s">
-        <v>43</v>
       </c>
       <c r="F13" s="10">
         <v>1</v>
@@ -5649,13 +5818,13 @@
         <v>28</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D14" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="E14" s="9" t="s">
         <v>42</v>
-      </c>
-      <c r="E14" s="9" t="s">
-        <v>43</v>
       </c>
       <c r="F14" s="10">
         <v>1</v>
@@ -5666,16 +5835,16 @@
         <v>13</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D15" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="E15" s="9" t="s">
         <v>42</v>
-      </c>
-      <c r="E15" s="9" t="s">
-        <v>43</v>
       </c>
       <c r="F15" s="10">
         <v>1</v>
@@ -5686,16 +5855,16 @@
         <v>14</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D16" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="E16" s="9" t="s">
         <v>42</v>
-      </c>
-      <c r="E16" s="9" t="s">
-        <v>43</v>
       </c>
       <c r="F16" s="10">
         <v>1</v>
@@ -5706,16 +5875,16 @@
         <v>15</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D17" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="E17" s="9" t="s">
         <v>42</v>
-      </c>
-      <c r="E17" s="9" t="s">
-        <v>43</v>
       </c>
       <c r="F17" s="10">
         <v>1</v>
@@ -5726,16 +5895,16 @@
         <v>16</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D18" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="E18" s="9" t="s">
         <v>42</v>
-      </c>
-      <c r="E18" s="9" t="s">
-        <v>43</v>
       </c>
       <c r="F18" s="10">
         <v>1</v>
@@ -5746,16 +5915,16 @@
         <v>17</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D19" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="E19" s="9" t="s">
         <v>42</v>
-      </c>
-      <c r="E19" s="9" t="s">
-        <v>43</v>
       </c>
       <c r="F19" s="10">
         <v>1</v>
@@ -5766,16 +5935,16 @@
         <v>18</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D20" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="E20" s="9" t="s">
         <v>42</v>
-      </c>
-      <c r="E20" s="9" t="s">
-        <v>43</v>
       </c>
       <c r="F20" s="10">
         <v>1</v>
@@ -5786,16 +5955,16 @@
         <v>19</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D21" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="E21" s="9" t="s">
         <v>42</v>
-      </c>
-      <c r="E21" s="9" t="s">
-        <v>43</v>
       </c>
       <c r="F21" s="10">
         <v>1</v>
@@ -5806,16 +5975,16 @@
         <v>20</v>
       </c>
       <c r="B22" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C22" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="D22" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="C22" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="D22" s="11" t="s">
+      <c r="E22" s="11" t="s">
         <v>42</v>
-      </c>
-      <c r="E22" s="11" t="s">
-        <v>43</v>
       </c>
       <c r="F22" s="12">
         <v>1</v>
@@ -5882,15 +6051,15 @@
   <sheetData>
     <row r="1" spans="1:2" ht="29.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="19" t="s">
         <v>44</v>
-      </c>
-      <c r="B1" s="19" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="29.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="20" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B2" s="21">
         <f>COUNTA(Raw_Data!B3:B22)</f>
@@ -5899,7 +6068,7 @@
     </row>
     <row r="3" spans="1:2" ht="29.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="20" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B3" s="21">
         <f>SUM(Raw_Data!F3:F22)</f>
@@ -5908,7 +6077,7 @@
     </row>
     <row r="4" spans="1:2" ht="29.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="20" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B4" s="21">
         <f>AVERAGE(Raw_Data!F3:F22)</f>
@@ -5917,7 +6086,7 @@
     </row>
     <row r="5" spans="1:2" ht="29.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="20" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B5" s="21">
         <f>MAX(Raw_Data!F3:F22)</f>
@@ -5926,7 +6095,7 @@
     </row>
     <row r="6" spans="1:2" ht="29.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="22" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B6" s="23">
         <f>MIN(Raw_Data!F3:F22)</f>
@@ -5951,16 +6120,16 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="34" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B1" s="34" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C1" s="8"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="35" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B2" s="35">
         <v>20</v>
@@ -5969,7 +6138,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="35" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B3" s="35">
         <v>27</v>
@@ -5978,7 +6147,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="35" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B4" s="35">
         <v>1.35</v>
@@ -5987,25 +6156,25 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="35" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B5" s="35" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C5" s="8"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="35" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B6" s="35" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C6" s="8"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="35" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B7" s="35" t="s">
         <v>23</v>
@@ -6014,7 +6183,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="35" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B8" s="35">
         <v>3</v>
@@ -6059,7 +6228,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="16" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B3" s="10">
         <f>SUMIF(Raw_Data!C:C,A3,Raw_Data!F:F)</f>
@@ -6068,7 +6237,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B4" s="10">
         <f>SUMIF(Raw_Data!C:C,A4,Raw_Data!F:F)</f>
@@ -6077,7 +6246,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B5" s="10">
         <f>SUMIF(Raw_Data!C:C,A5,Raw_Data!F:F)</f>
@@ -6086,7 +6255,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B6" s="10">
         <f>SUMIF(Raw_Data!C:C,A6,Raw_Data!F:F)</f>
@@ -6095,7 +6264,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" s="16" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B7" s="10">
         <f>SUMIF(Raw_Data!C:C,A7,Raw_Data!F:F)</f>
@@ -6104,7 +6273,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" s="16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B8" s="10">
         <f>SUMIF(Raw_Data!C:C,A8,Raw_Data!F:F)</f>
@@ -6113,7 +6282,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" s="16" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B9" s="10">
         <f>SUMIF(Raw_Data!C:C,A9,Raw_Data!F:F)</f>
@@ -6122,7 +6291,7 @@
     </row>
     <row r="10" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="17" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B10" s="12">
         <f>SUMIF(Raw_Data!C:C,A10,Raw_Data!F:F)</f>
@@ -6147,15 +6316,15 @@
   <sheetData>
     <row r="1" spans="1:8" ht="18.5" x14ac:dyDescent="0.35">
       <c r="A1" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" s="27" t="s">
         <v>60</v>
-      </c>
-      <c r="B1" s="27" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="26" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B2" s="26">
         <v>10</v>
@@ -6163,22 +6332,22 @@
     </row>
     <row r="3" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="26" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B3" s="26">
         <v>8</v>
       </c>
-      <c r="D3" s="42" t="s">
-        <v>69</v>
-      </c>
-      <c r="E3" s="43"/>
-      <c r="F3" s="43"/>
-      <c r="G3" s="43"/>
-      <c r="H3" s="43"/>
+      <c r="D3" s="59" t="s">
+        <v>68</v>
+      </c>
+      <c r="E3" s="60"/>
+      <c r="F3" s="60"/>
+      <c r="G3" s="60"/>
+      <c r="H3" s="60"/>
     </row>
     <row r="4" spans="1:8" ht="21.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="26" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B4" s="26">
         <v>4</v>
@@ -6186,7 +6355,7 @@
     </row>
     <row r="5" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="26" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B5" s="26">
         <v>3</v>
@@ -6194,7 +6363,7 @@
     </row>
     <row r="6" spans="1:8" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="26" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B6" s="26">
         <v>2</v>
@@ -6207,7 +6376,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B14" s="8">
         <f>-SUM(B2:B6)</f>
@@ -6220,7 +6389,7 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B16" s="8" t="str">
         <f>INDEX(A2:A6,MATCH(MAX(B2:B6),B2:B6,0))</f>
@@ -6251,116 +6420,116 @@
   <sheetData>
     <row r="1" spans="1:19" ht="22" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="28" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B1" s="29" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="21" x14ac:dyDescent="0.5">
       <c r="A2" s="30" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B2" s="31">
         <f>SUM('Performance overview'!B2)</f>
         <v>20</v>
       </c>
-      <c r="G2" s="44" t="s">
-        <v>75</v>
-      </c>
-      <c r="H2" s="44"/>
-      <c r="I2" s="44"/>
-      <c r="J2" s="44"/>
-      <c r="K2" s="44"/>
-      <c r="O2" s="45" t="s">
-        <v>77</v>
-      </c>
-      <c r="P2" s="46"/>
-      <c r="Q2" s="46"/>
-      <c r="R2" s="46"/>
-      <c r="S2" s="47"/>
+      <c r="G2" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="H2" s="61"/>
+      <c r="I2" s="61"/>
+      <c r="J2" s="61"/>
+      <c r="K2" s="61"/>
+      <c r="O2" s="62" t="s">
+        <v>76</v>
+      </c>
+      <c r="P2" s="63"/>
+      <c r="Q2" s="63"/>
+      <c r="R2" s="63"/>
+      <c r="S2" s="64"/>
     </row>
     <row r="3" spans="1:19" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A3" s="30" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B3" s="31">
         <f>SUM('Performance overview'!B3)</f>
         <v>27</v>
       </c>
-      <c r="O3" s="48" t="s">
-        <v>78</v>
-      </c>
-      <c r="P3" s="49"/>
-      <c r="Q3" s="49"/>
-      <c r="R3" s="49"/>
-      <c r="S3" s="50"/>
+      <c r="O3" s="65" t="s">
+        <v>77</v>
+      </c>
+      <c r="P3" s="66"/>
+      <c r="Q3" s="66"/>
+      <c r="R3" s="66"/>
+      <c r="S3" s="67"/>
     </row>
     <row r="4" spans="1:19" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A4" s="30" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B4" s="31">
         <f>MAX(category_Analysis!A1:C10)</f>
         <v>9</v>
       </c>
-      <c r="O4" s="48" t="s">
-        <v>79</v>
-      </c>
-      <c r="P4" s="49"/>
-      <c r="Q4" s="49"/>
-      <c r="R4" s="49"/>
-      <c r="S4" s="50"/>
+      <c r="O4" s="65" t="s">
+        <v>78</v>
+      </c>
+      <c r="P4" s="66"/>
+      <c r="Q4" s="66"/>
+      <c r="R4" s="66"/>
+      <c r="S4" s="67"/>
     </row>
     <row r="5" spans="1:19" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A5" s="30" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B5" s="31">
         <f>MAX(Hook_Analysis!A1:B6)</f>
         <v>10</v>
       </c>
-      <c r="O5" s="48" t="s">
-        <v>80</v>
-      </c>
-      <c r="P5" s="49"/>
-      <c r="Q5" s="49"/>
-      <c r="R5" s="49"/>
-      <c r="S5" s="50"/>
+      <c r="O5" s="65" t="s">
+        <v>79</v>
+      </c>
+      <c r="P5" s="66"/>
+      <c r="Q5" s="66"/>
+      <c r="R5" s="66"/>
+      <c r="S5" s="67"/>
     </row>
     <row r="6" spans="1:19" ht="19" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A6" s="32" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B6" s="33">
         <f>AVERAGE('Performance overview'!B4)</f>
         <v>1.35</v>
       </c>
-      <c r="O6" s="48" t="s">
+      <c r="O6" s="65" t="s">
+        <v>80</v>
+      </c>
+      <c r="P6" s="66"/>
+      <c r="Q6" s="66"/>
+      <c r="R6" s="66"/>
+      <c r="S6" s="67"/>
+    </row>
+    <row r="7" spans="1:19" ht="19" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="O7" s="68" t="s">
         <v>81</v>
       </c>
-      <c r="P6" s="49"/>
-      <c r="Q6" s="49"/>
-      <c r="R6" s="49"/>
-      <c r="S6" s="50"/>
-    </row>
-    <row r="7" spans="1:19" ht="19" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="O7" s="51" t="s">
-        <v>82</v>
-      </c>
-      <c r="P7" s="52"/>
-      <c r="Q7" s="52"/>
-      <c r="R7" s="52"/>
-      <c r="S7" s="53"/>
+      <c r="P7" s="69"/>
+      <c r="Q7" s="69"/>
+      <c r="R7" s="69"/>
+      <c r="S7" s="70"/>
     </row>
     <row r="22" spans="7:11" ht="21" x14ac:dyDescent="0.5">
-      <c r="G22" s="44" t="s">
-        <v>76</v>
-      </c>
-      <c r="H22" s="44"/>
-      <c r="I22" s="44"/>
-      <c r="J22" s="44"/>
-      <c r="K22" s="44"/>
+      <c r="G22" s="61" t="s">
+        <v>75</v>
+      </c>
+      <c r="H22" s="61"/>
+      <c r="I22" s="61"/>
+      <c r="J22" s="61"/>
+      <c r="K22" s="61"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -6394,10 +6563,10 @@
         <v>16</v>
       </c>
       <c r="C1" s="36" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D1" s="38" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
@@ -6405,7 +6574,7 @@
         <v>23</v>
       </c>
       <c r="B2" s="37" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C2" s="37">
         <v>3</v>
@@ -6420,7 +6589,7 @@
         <v>24</v>
       </c>
       <c r="B3" s="37" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C3" s="37">
         <v>3</v>
@@ -6435,7 +6604,7 @@
         <v>25</v>
       </c>
       <c r="B4" s="37" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C4" s="37">
         <v>2</v>
@@ -6447,10 +6616,10 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="37" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B5" s="37" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C5" s="37">
         <v>2</v>
@@ -6462,10 +6631,10 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="37" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B6" s="37" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C6" s="37">
         <v>2</v>
@@ -6480,7 +6649,7 @@
         <v>28</v>
       </c>
       <c r="B7" s="37" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C7" s="37">
         <v>1</v>
@@ -6492,10 +6661,10 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="37" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B8" s="37" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C8" s="37">
         <v>1</v>
@@ -6507,10 +6676,10 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="37" t="s">
+        <v>91</v>
+      </c>
+      <c r="B9" s="37" t="s">
         <v>92</v>
-      </c>
-      <c r="B9" s="37" t="s">
-        <v>93</v>
       </c>
       <c r="C9" s="37">
         <v>1</v>
@@ -6521,90 +6690,90 @@
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A13" s="54" t="s">
-        <v>97</v>
-      </c>
-      <c r="B13" s="54"/>
+      <c r="A13" s="71" t="s">
+        <v>96</v>
+      </c>
+      <c r="B13" s="71"/>
       <c r="C13">
         <f>COUNTIF(C2:C9,1)</f>
         <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A14" s="54" t="s">
-        <v>98</v>
-      </c>
-      <c r="B14" s="54"/>
+      <c r="A14" s="71" t="s">
+        <v>97</v>
+      </c>
+      <c r="B14" s="71"/>
       <c r="C14">
         <f>COUNTIF(D2:D9,"Good")</f>
         <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="54" t="s">
-        <v>99</v>
-      </c>
-      <c r="B15" s="54"/>
+      <c r="A15" s="71" t="s">
+        <v>98</v>
+      </c>
+      <c r="B15" s="71"/>
       <c r="C15">
         <f>(SUMIF(B2:B9,"Home Organization",C2:C9))</f>
         <v>6</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A16" s="54" t="s">
-        <v>100</v>
-      </c>
-      <c r="B16" s="54"/>
+      <c r="A16" s="71" t="s">
+        <v>99</v>
+      </c>
+      <c r="B16" s="71"/>
       <c r="C16">
         <f>AVERAGEIF(B2:B9,"School",C2:C9)</f>
         <v>1.6666666666666667</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A20" s="54" t="s">
-        <v>101</v>
-      </c>
-      <c r="B20" s="54"/>
+      <c r="A20" s="71" t="s">
+        <v>100</v>
+      </c>
+      <c r="B20" s="71"/>
       <c r="C20">
         <f>COUNTIF(B2:B9,"School")</f>
         <v>3</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A21" s="54" t="s">
-        <v>102</v>
-      </c>
-      <c r="B21" s="54"/>
+      <c r="A21" s="71" t="s">
+        <v>101</v>
+      </c>
+      <c r="B21" s="71"/>
       <c r="C21">
         <f>COUNTIF(B2:B9,"Home Organization")</f>
         <v>3</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A22" s="54" t="s">
-        <v>103</v>
-      </c>
-      <c r="B22" s="54"/>
+      <c r="A22" s="71" t="s">
+        <v>102</v>
+      </c>
+      <c r="B22" s="71"/>
       <c r="C22">
         <f>SUMIF(B2:B9,"Kitchen",C2:C9)</f>
         <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A23" s="54" t="s">
-        <v>104</v>
-      </c>
-      <c r="B23" s="54"/>
+      <c r="A23" s="71" t="s">
+        <v>103</v>
+      </c>
+      <c r="B23" s="71"/>
       <c r="C23">
         <f>AVERAGEIF(B2:B9,"Home Organization",C2:C9)</f>
         <v>2</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A24" s="54" t="s">
-        <v>105</v>
-      </c>
-      <c r="B24" s="54"/>
+      <c r="A24" s="71" t="s">
+        <v>104</v>
+      </c>
+      <c r="B24" s="71"/>
       <c r="C24">
         <f>COUNTIF(D2:D9,"low")</f>
         <v>3</v>
@@ -6642,39 +6811,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A1" s="56" t="s">
-        <v>116</v>
-      </c>
-      <c r="B1" s="57" t="s">
+      <c r="A1" s="40" t="s">
+        <v>115</v>
+      </c>
+      <c r="B1" s="41" t="s">
+        <v>117</v>
+      </c>
+      <c r="C1" s="41" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="41" t="s">
+        <v>105</v>
+      </c>
+      <c r="E1" s="42" t="s">
         <v>118</v>
       </c>
-      <c r="C1" s="57" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1" s="57" t="s">
+      <c r="G1" s="48" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A2" s="43" t="s">
         <v>106</v>
       </c>
-      <c r="E1" s="58" t="s">
+      <c r="B2" s="39" t="s">
         <v>119</v>
       </c>
-      <c r="G1" s="64" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" s="59" t="s">
-        <v>107</v>
-      </c>
-      <c r="B2" s="55" t="s">
-        <v>120</v>
-      </c>
-      <c r="C2" s="55" t="s">
-        <v>114</v>
-      </c>
-      <c r="D2" s="55">
+      <c r="C2" s="39" t="s">
+        <v>113</v>
+      </c>
+      <c r="D2" s="39">
         <v>80</v>
       </c>
-      <c r="E2" s="60">
+      <c r="E2" s="44">
         <v>25</v>
       </c>
       <c r="G2" t="str">
@@ -6683,19 +6852,19 @@
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" s="59" t="s">
-        <v>108</v>
-      </c>
-      <c r="B3" s="55" t="s">
-        <v>121</v>
-      </c>
-      <c r="C3" s="55" t="s">
-        <v>114</v>
-      </c>
-      <c r="D3" s="55">
+      <c r="A3" s="43" t="s">
+        <v>107</v>
+      </c>
+      <c r="B3" s="39" t="s">
         <v>120</v>
       </c>
-      <c r="E3" s="60">
+      <c r="C3" s="39" t="s">
+        <v>113</v>
+      </c>
+      <c r="D3" s="39">
+        <v>120</v>
+      </c>
+      <c r="E3" s="44">
         <v>40</v>
       </c>
       <c r="G3">
@@ -6704,19 +6873,19 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" s="59" t="s">
-        <v>109</v>
-      </c>
-      <c r="B4" s="55" t="s">
-        <v>112</v>
-      </c>
-      <c r="C4" s="55" t="s">
-        <v>123</v>
-      </c>
-      <c r="D4" s="55">
+      <c r="A4" s="43" t="s">
+        <v>108</v>
+      </c>
+      <c r="B4" s="39" t="s">
+        <v>111</v>
+      </c>
+      <c r="C4" s="39" t="s">
+        <v>122</v>
+      </c>
+      <c r="D4" s="39">
         <v>250</v>
       </c>
-      <c r="E4" s="60">
+      <c r="E4" s="44">
         <v>15</v>
       </c>
       <c r="G4">
@@ -6725,19 +6894,19 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5" s="59" t="s">
-        <v>110</v>
-      </c>
-      <c r="B5" s="55" t="s">
-        <v>113</v>
-      </c>
-      <c r="C5" s="55" t="s">
-        <v>123</v>
-      </c>
-      <c r="D5" s="55">
+      <c r="A5" s="43" t="s">
+        <v>109</v>
+      </c>
+      <c r="B5" s="39" t="s">
+        <v>112</v>
+      </c>
+      <c r="C5" s="39" t="s">
+        <v>122</v>
+      </c>
+      <c r="D5" s="39">
         <v>600</v>
       </c>
-      <c r="E5" s="60">
+      <c r="E5" s="44">
         <v>10</v>
       </c>
       <c r="G5" t="str">
@@ -6746,19 +6915,19 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" s="59" t="s">
-        <v>111</v>
-      </c>
-      <c r="B6" s="55" t="s">
-        <v>122</v>
-      </c>
-      <c r="C6" s="55" t="s">
-        <v>124</v>
-      </c>
-      <c r="D6" s="55">
+      <c r="A6" s="43" t="s">
+        <v>110</v>
+      </c>
+      <c r="B6" s="39" t="s">
+        <v>121</v>
+      </c>
+      <c r="C6" s="39" t="s">
+        <v>123</v>
+      </c>
+      <c r="D6" s="39">
         <v>450</v>
       </c>
-      <c r="E6" s="60">
+      <c r="E6" s="44">
         <v>20</v>
       </c>
       <c r="G6">
@@ -6767,19 +6936,19 @@
       </c>
     </row>
     <row r="7" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="61" t="s">
-        <v>117</v>
-      </c>
-      <c r="B7" s="62" t="s">
-        <v>92</v>
-      </c>
-      <c r="C7" s="62" t="s">
-        <v>124</v>
-      </c>
-      <c r="D7" s="62">
+      <c r="A7" s="45" t="s">
+        <v>116</v>
+      </c>
+      <c r="B7" s="46" t="s">
+        <v>91</v>
+      </c>
+      <c r="C7" s="46" t="s">
+        <v>123</v>
+      </c>
+      <c r="D7" s="46">
         <v>300</v>
       </c>
-      <c r="E7" s="63">
+      <c r="E7" s="47">
         <v>30</v>
       </c>
       <c r="G7">

</xml_diff>